<commit_message>
Documenti PPR: generazione dal template MOD-PPR via Excel
- Cover sempre dal nuovo template (incluso Independent Reviewer), nomi per ruolo dal documento precedente secondo applicabilita' del template; con documento precedente su vecchio template si prendono solo versione e Revision History
- Meeting Attendees and Roles riportati dal meeting precedente, segnaposto arancioni rimossi salvo Independent Reviewer mancante
- File <Fase>-review-documents.txt per Execution, Deployment e Release to Market con documenti del Deliverable Check e owner dal Task Guideline, scaricabile dal popup di conferma
- Popup di caricamento con tipo di documento piu' evidente

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/app/templates/ppr_template.xlsx
+++ b/backend/app/templates/ppr_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inpeco-my.sharepoint.com/personal/luca_contini_inpeco_com/Documents/Projects/ProTube System Project/PTBSYS-03-003 - October/Reviews and Technical Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9EF4B58-F2B1-4862-9A4E-41761AC4DC64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4DBDA00-54D5-4197-95F8-1F68BD4FE087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="779" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="779" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Task Guideline" sheetId="22" r:id="rId1"/>
@@ -13190,7 +13190,7 @@
     <mergeCell ref="G12:K12"/>
   </mergeCells>
   <pageMargins left="0.65833333333333333" right="0.59166666666666667" top="0.96666666666666667" bottom="1.0333333333333334" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="78" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="77" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;G&amp;C&amp;"Montserrat,Bold"&amp;12&amp;K00B4E4Cover&amp;R&amp;"Montserrat,Bold"&amp;12&amp;K00B4E4Project Phase Review</oddHeader>
     <oddFooter>&amp;L&amp;"Montserrat,Regular"&amp;9&amp;K333333MOD-PPR.1&amp;KFF0000
@@ -15175,7 +15175,7 @@
     <mergeCell ref="F11:J11"/>
   </mergeCells>
   <pageMargins left="0.65833333333333333" right="0.59166666666666667" top="0.96666666666666667" bottom="1.0333333333333334" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="67" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="66" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader xml:space="preserve">&amp;L&amp;G&amp;C&amp;"Montserrat,Bold"&amp;12&amp;K00B4E4Pre-Serie Launch Review&amp;R&amp;"Montserrat,Bold"&amp;12&amp;K00B4E4Project Phase Review     </oddHeader>
     <oddFooter>&amp;L&amp;"Montserrat,Regular"&amp;10MOD-PPR.1

</xml_diff>